<commit_message>
Changes in heat map files
</commit_message>
<xml_diff>
--- a/data/Heat map 6.xlsx
+++ b/data/Heat map 6.xlsx
@@ -1,19 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F74C27BE-7312-4C26-BAC3-DEABC6EF9CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{76F2D5A9-3AE0-44CD-930A-817A40FC2D01}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Reputation, Society" sheetId="1" r:id="rId1"/>
+    <sheet name="Reputation, Society" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
@@ -22,223 +15,114 @@
     <definedName name="_Hlk200085589" localSheetId="0">'Reputation, Society'!#REF!</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Reputation, Society'!$B$1:$L$17</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
-  <si>
-    <t>KPI by FTE</t>
-  </si>
-  <si>
-    <t>Recognition and Reputation</t>
-  </si>
-  <si>
-    <t>Society Impact &amp; Inclusion</t>
-  </si>
-  <si>
-    <t>Number of collaborations with ARIs</t>
-  </si>
-  <si>
-    <t>Number of active collaborations with scaling partners</t>
-  </si>
-  <si>
-    <t>Number of awards granted to IITA staff/project teams</t>
-  </si>
-  <si>
-    <t>Number of invitations to IITA staff to give seminars, as guest speakers etc.</t>
-  </si>
-  <si>
-    <t>Number of direct engagements  with senior policymakers to provide strategic advice, influence reforms, or shape national strategies.</t>
-  </si>
-  <si>
-    <t>Approved proposals with gender/youth/social inclusion components (target is 25% of total approved proposals)</t>
-  </si>
-  <si>
-    <t>Approved proposals with inclusion of adaptation/ mitigation activities  (target is 25% of total approved proposals)</t>
-  </si>
-  <si>
-    <t>Approved proposals with inclusion of nutrition and health activities (target is 25% of total approved proposals)</t>
-  </si>
-  <si>
-    <t>GI</t>
-  </si>
-  <si>
-    <t>Biotech</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Breeding</t>
-  </si>
-  <si>
-    <t>Genebanks</t>
-  </si>
-  <si>
-    <t>Seed System</t>
-  </si>
-  <si>
-    <t>RAFS</t>
-  </si>
-  <si>
-    <t>Plant Health</t>
-  </si>
-  <si>
-    <t>Farming Systems Agronomy</t>
-  </si>
-  <si>
-    <t>NRM</t>
-  </si>
-  <si>
-    <t>Mechanization</t>
-  </si>
-  <si>
-    <t>ST</t>
-  </si>
-  <si>
-    <t>FIAS</t>
-  </si>
-  <si>
-    <t>GeYSI</t>
-  </si>
-  <si>
-    <t>RCA</t>
-  </si>
-  <si>
-    <t>Nutrition</t>
-  </si>
-  <si>
-    <t>VCMA</t>
-  </si>
-  <si>
-    <t>per Program Target (target/13)</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="12">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="9"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF0070C0"/>
+      <sz val="9"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF00B0F0"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FFFF0000"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="8"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="9"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF0070C0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF0070C0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <fgColor theme="2" tint="-0.09997863704336681"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -739,242 +623,407 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF00B050"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="92">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
+<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook r:id="rId1">
     <sheetNames>
       <sheetName val="Chart1"/>
       <sheetName val="Sheet1"/>
@@ -1371,580 +1420,644 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D64F6B4-64C6-41A0-9F63-399977D02850}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AB23"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:AB21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="3.21875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" style="1" customWidth="1"/>
-    <col min="4" max="10" width="8.5546875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5546875" style="28" customWidth="1"/>
-    <col min="12" max="12" width="5.44140625" style="28" customWidth="1"/>
-    <col min="13" max="14" width="8.21875" style="3" customWidth="1"/>
+    <col width="3.21875" customWidth="1" style="1" min="2" max="2"/>
+    <col width="25.33203125" customWidth="1" style="1" min="3" max="3"/>
+    <col width="8.5546875" customWidth="1" style="1" min="4" max="10"/>
+    <col width="8.5546875" customWidth="1" style="74" min="11" max="11"/>
+    <col width="5.44140625" customWidth="1" style="74" min="12" max="12"/>
+    <col width="8.21875" customWidth="1" style="75" min="13" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="15" thickBot="1">
-      <c r="C1" s="65" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="2"/>
+    <row r="1" ht="15" customHeight="1" thickBot="1">
+      <c r="C1" s="65" t="inlineStr">
+        <is>
+          <t>KPI by FTE</t>
+        </is>
+      </c>
+      <c r="D1" s="76" t="n"/>
+      <c r="E1" s="76" t="n"/>
+      <c r="F1" s="76" t="n"/>
+      <c r="G1" s="76" t="n"/>
+      <c r="H1" s="76" t="n"/>
+      <c r="I1" s="76" t="n"/>
+      <c r="J1" s="76" t="n"/>
+      <c r="K1" s="77" t="n"/>
+      <c r="L1" s="78" t="n"/>
     </row>
-    <row r="2" spans="2:14" s="8" customFormat="1" ht="25.95" customHeight="1" thickBot="1">
-      <c r="B2" s="4"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="72" t="s">
-        <v>2</v>
-      </c>
-      <c r="J2" s="72"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
+    <row r="2" ht="25.95" customFormat="1" customHeight="1" s="8" thickBot="1">
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="69" t="inlineStr">
+        <is>
+          <t>Recognition and Reputation</t>
+        </is>
+      </c>
+      <c r="E2" s="79" t="n"/>
+      <c r="F2" s="79" t="n"/>
+      <c r="G2" s="79" t="n"/>
+      <c r="H2" s="80" t="n"/>
+      <c r="I2" s="73" t="inlineStr">
+        <is>
+          <t>Society Impact &amp; Inclusion</t>
+        </is>
+      </c>
+      <c r="J2" s="76" t="n"/>
+      <c r="K2" s="81" t="n"/>
+      <c r="L2" s="82" t="n"/>
+      <c r="M2" s="83" t="n"/>
+      <c r="N2" s="83" t="n"/>
     </row>
-    <row r="3" spans="2:14" s="18" customFormat="1" ht="132" customHeight="1" thickBot="1">
-      <c r="B3" s="9"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="J3" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="K3" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="L3" s="2"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="17"/>
+    <row r="3" ht="132" customFormat="1" customHeight="1" s="18" thickBot="1">
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>ARIs collaborations</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Active collaborations with scaling partners</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>Awards grated to IITA stafff</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>Invitations to give seminars/talks</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>High level engagements</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>Approved proposals with GeYSI components</t>
+        </is>
+      </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>Approved proposals with climate components</t>
+        </is>
+      </c>
+      <c r="K3" s="16" t="inlineStr">
+        <is>
+          <t>Approved proposals with nutrition and health components</t>
+        </is>
+      </c>
+      <c r="L3" s="78" t="n"/>
+      <c r="M3" s="84" t="n"/>
+      <c r="N3" s="84" t="n"/>
     </row>
-    <row r="4" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B4" s="59" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="20">
-        <v>2.4285714285714284</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>13</v>
+    <row r="4" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B4" s="59" t="inlineStr">
+        <is>
+          <t>GI</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>Biotech</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="n">
+        <v>2.428571428571428</v>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="F4" s="22">
         <f>[1]Sheet1!$U$18</f>
-        <v>0.14285714285714285</v>
-      </c>
-      <c r="G4" s="23">
-        <v>0</v>
-      </c>
-      <c r="H4" s="24"/>
-      <c r="I4" s="25">
-        <v>0</v>
-      </c>
-      <c r="J4" s="26">
-        <v>0</v>
-      </c>
-      <c r="K4" s="27">
-        <v>0</v>
-      </c>
-      <c r="L4" s="2"/>
-      <c r="M4" s="28"/>
-      <c r="N4" s="28"/>
+        <v/>
+      </c>
+      <c r="G4" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="24" t="n"/>
+      <c r="I4" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="78" t="n"/>
+      <c r="M4" s="74" t="n"/>
+      <c r="N4" s="74" t="n"/>
     </row>
-    <row r="5" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B5" s="60"/>
-      <c r="C5" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="20">
+    <row r="5" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B5" s="85" t="n"/>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Breeding</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="22">
-        <v>0</v>
-      </c>
-      <c r="G5" s="23">
-        <v>0.13043478260869565</v>
-      </c>
-      <c r="H5" s="24"/>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>0.1304347826086956</v>
+      </c>
+      <c r="H5" s="24" t="n"/>
       <c r="I5" s="31">
         <f>[1]Sheet1!$W$21</f>
-        <v>8.6956521739130432E-2</v>
+        <v/>
       </c>
       <c r="J5" s="32">
         <f>[1]Sheet1!$W$22</f>
-        <v>4.3478260869565216E-2</v>
+        <v/>
       </c>
       <c r="K5" s="24">
         <f>[1]Sheet1!$W$23</f>
-        <v>8.6956521739130432E-2</v>
-      </c>
-      <c r="L5" s="2"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
+        <v/>
+      </c>
+      <c r="L5" s="78" t="n"/>
+      <c r="M5" s="74" t="n"/>
+      <c r="N5" s="74" t="n"/>
     </row>
-    <row r="6" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B6" s="60"/>
-      <c r="C6" s="30" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="20">
+    <row r="6" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B6" s="85" t="n"/>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>Genebanks</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="n">
         <v>4.75</v>
       </c>
-      <c r="E6" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="22">
-        <v>0</v>
-      </c>
-      <c r="G6" s="23">
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="23" t="n">
         <v>0.25</v>
       </c>
-      <c r="H6" s="24"/>
-      <c r="I6" s="31">
-        <v>0</v>
-      </c>
-      <c r="J6" s="32">
-        <v>0</v>
-      </c>
-      <c r="K6" s="24">
-        <v>0</v>
-      </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
+      <c r="H6" s="24" t="n"/>
+      <c r="I6" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="78" t="n"/>
+      <c r="M6" s="74" t="n"/>
+      <c r="N6" s="74" t="n"/>
     </row>
-    <row r="7" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B7" s="61"/>
-      <c r="C7" s="33" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="20">
-        <v>0</v>
-      </c>
-      <c r="E7" s="21">
-        <v>0.93333333333333335</v>
+    <row r="7" ht="15.6" customFormat="1" customHeight="1" s="29" thickBot="1">
+      <c r="B7" s="86" t="n"/>
+      <c r="C7" s="33" t="inlineStr">
+        <is>
+          <t>Seed System</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>0.9333333333333333</v>
       </c>
       <c r="F7" s="22">
         <f>[1]Sheet1!$AA$18</f>
-        <v>0.2</v>
-      </c>
-      <c r="G7" s="23">
-        <v>0</v>
-      </c>
-      <c r="H7" s="24"/>
+        <v/>
+      </c>
+      <c r="G7" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="24" t="n"/>
       <c r="I7" s="34">
         <f>[1]Sheet1!$AA$21</f>
-        <v>0.2</v>
+        <v/>
       </c>
       <c r="J7" s="35">
         <f>[1]Sheet1!$AA$22</f>
-        <v>0.13333333333333333</v>
+        <v/>
       </c>
       <c r="K7" s="36">
         <f>[1]Sheet1!$AA$23</f>
-        <v>6.6666666666666666E-2</v>
-      </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="28"/>
-      <c r="N7" s="28"/>
+        <v/>
+      </c>
+      <c r="L7" s="78" t="n"/>
+      <c r="M7" s="74" t="n"/>
+      <c r="N7" s="74" t="n"/>
     </row>
-    <row r="8" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B8" s="59" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="20">
+    <row r="8" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B8" s="59" t="inlineStr">
+        <is>
+          <t>RAFS</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Plant Health</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="n">
         <v>1.5</v>
       </c>
-      <c r="E8" s="21">
-        <v>8.3333333333333329E-2</v>
+      <c r="E8" s="21" t="n">
+        <v>0.08333333333333333</v>
       </c>
       <c r="F8" s="22">
         <f>[1]Sheet1!$AC$18</f>
-        <v>0.25</v>
-      </c>
-      <c r="G8" s="23">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="H8" s="24"/>
+        <v/>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H8" s="24" t="n"/>
       <c r="I8" s="25">
         <f>[1]Sheet1!$AC$21</f>
-        <v>8.3333333333333329E-2</v>
+        <v/>
       </c>
       <c r="J8" s="26">
         <f>[1]Sheet1!$AC$22</f>
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="K8" s="27">
-        <v>0</v>
-      </c>
-      <c r="L8" s="2"/>
-      <c r="M8" s="28"/>
-      <c r="N8" s="28"/>
+        <v/>
+      </c>
+      <c r="K8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="78" t="n"/>
+      <c r="M8" s="74" t="n"/>
+      <c r="N8" s="74" t="n"/>
     </row>
-    <row r="9" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B9" s="60"/>
-      <c r="C9" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="20">
+    <row r="9" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B9" s="85" t="n"/>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>Farming Systems Agronomy</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="n">
         <v>2.15</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="21" t="n">
         <v>0.85</v>
       </c>
-      <c r="F9" s="22">
-        <v>0</v>
-      </c>
-      <c r="G9" s="23">
+      <c r="F9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="23" t="n">
         <v>0.15</v>
       </c>
-      <c r="H9" s="24"/>
+      <c r="H9" s="24" t="n"/>
       <c r="I9" s="31">
         <f>[1]Sheet1!$AE$21</f>
-        <v>0.2</v>
+        <v/>
       </c>
       <c r="J9" s="32">
         <f>[1]Sheet1!$AE$22</f>
-        <v>0.2</v>
+        <v/>
       </c>
       <c r="K9" s="24">
         <f>[1]Sheet1!$AE$23</f>
-        <v>0.05</v>
-      </c>
-      <c r="L9" s="2"/>
-      <c r="M9" s="28"/>
-      <c r="N9" s="28"/>
+        <v/>
+      </c>
+      <c r="L9" s="78" t="n"/>
+      <c r="M9" s="74" t="n"/>
+      <c r="N9" s="74" t="n"/>
     </row>
-    <row r="10" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B10" s="60"/>
-      <c r="C10" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="20">
-        <v>0</v>
-      </c>
-      <c r="E10" s="21">
-        <v>0.42857142857142855</v>
-      </c>
-      <c r="F10" s="22">
-        <v>0</v>
-      </c>
-      <c r="G10" s="23">
-        <v>0</v>
-      </c>
-      <c r="H10" s="24"/>
+    <row r="10" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B10" s="85" t="n"/>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>NRM</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="24" t="n"/>
       <c r="I10" s="31">
         <f>[1]Sheet1!$AG$21</f>
-        <v>0.5714285714285714</v>
+        <v/>
       </c>
       <c r="J10" s="32">
         <f>[1]Sheet1!$AG$22</f>
-        <v>0.7142857142857143</v>
-      </c>
-      <c r="K10" s="24">
-        <v>0</v>
-      </c>
-      <c r="L10" s="2"/>
-      <c r="M10" s="28"/>
-      <c r="N10" s="28"/>
+        <v/>
+      </c>
+      <c r="K10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="78" t="n"/>
+      <c r="M10" s="74" t="n"/>
+      <c r="N10" s="74" t="n"/>
     </row>
-    <row r="11" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B11" s="61"/>
-      <c r="C11" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="20">
-        <v>0</v>
-      </c>
-      <c r="E11" s="21">
-        <v>0</v>
-      </c>
-      <c r="F11" s="22">
-        <v>0</v>
-      </c>
-      <c r="G11" s="23">
-        <v>0</v>
-      </c>
-      <c r="H11" s="24"/>
-      <c r="I11" s="34">
-        <v>0</v>
-      </c>
-      <c r="J11" s="35">
-        <v>0</v>
-      </c>
-      <c r="K11" s="36">
-        <v>0</v>
-      </c>
-      <c r="L11" s="2"/>
-      <c r="M11" s="28"/>
-      <c r="N11" s="28"/>
+    <row r="11" ht="15.6" customFormat="1" customHeight="1" s="29" thickBot="1">
+      <c r="B11" s="86" t="n"/>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>Mechanization</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="24" t="n"/>
+      <c r="I11" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="78" t="n"/>
+      <c r="M11" s="74" t="n"/>
+      <c r="N11" s="74" t="n"/>
     </row>
-    <row r="12" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B12" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="D12" s="20">
-        <v>0.63636363636363635</v>
-      </c>
-      <c r="E12" s="21">
-        <v>0</v>
-      </c>
-      <c r="F12" s="22">
-        <v>0</v>
-      </c>
-      <c r="G12" s="39">
-        <v>0</v>
-      </c>
-      <c r="H12" s="24"/>
-      <c r="I12" s="40">
-        <v>0</v>
-      </c>
-      <c r="J12" s="41">
-        <v>0</v>
-      </c>
-      <c r="K12" s="42">
-        <v>0</v>
-      </c>
-      <c r="L12" s="2"/>
-      <c r="M12" s="28"/>
-      <c r="N12" s="28"/>
+    <row r="12" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B12" s="87" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="inlineStr">
+        <is>
+          <t>FIAS</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="n">
+        <v>0.6363636363636364</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="24" t="n"/>
+      <c r="I12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="78" t="n"/>
+      <c r="M12" s="74" t="n"/>
+      <c r="N12" s="74" t="n"/>
     </row>
-    <row r="13" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B13" s="63"/>
-      <c r="C13" s="37" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="20">
-        <v>0</v>
-      </c>
-      <c r="E13" s="21">
-        <v>0</v>
-      </c>
-      <c r="F13" s="22">
-        <v>0</v>
-      </c>
-      <c r="G13" s="39">
-        <v>0.27272727272727271</v>
-      </c>
-      <c r="H13" s="24"/>
-      <c r="I13" s="43">
-        <v>0</v>
-      </c>
-      <c r="J13" s="32">
-        <v>0</v>
-      </c>
-      <c r="K13" s="24">
-        <v>0</v>
-      </c>
-      <c r="L13" s="2"/>
-      <c r="M13" s="28"/>
-      <c r="N13" s="28"/>
+    <row r="13" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B13" s="85" t="n"/>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>GeYSI</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="39" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="H13" s="24" t="n"/>
+      <c r="I13" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="78" t="n"/>
+      <c r="M13" s="74" t="n"/>
+      <c r="N13" s="74" t="n"/>
     </row>
-    <row r="14" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B14" s="63"/>
-      <c r="C14" s="37" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" s="20">
+    <row r="14" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B14" s="85" t="n"/>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>RCA</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="n">
         <v>1.2</v>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="21" t="n">
         <v>0.6</v>
       </c>
-      <c r="F14" s="22">
-        <v>0</v>
-      </c>
-      <c r="G14" s="39">
+      <c r="F14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="39" t="n">
         <v>0.6</v>
       </c>
-      <c r="H14" s="24"/>
-      <c r="I14" s="43">
-        <v>0</v>
-      </c>
-      <c r="J14" s="32">
-        <v>0</v>
-      </c>
-      <c r="K14" s="24">
-        <v>0</v>
-      </c>
-      <c r="L14" s="2"/>
-      <c r="M14" s="28"/>
-      <c r="N14" s="28"/>
+      <c r="H14" s="24" t="n"/>
+      <c r="I14" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="78" t="n"/>
+      <c r="M14" s="74" t="n"/>
+      <c r="N14" s="74" t="n"/>
     </row>
-    <row r="15" spans="2:14" s="29" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B15" s="63"/>
-      <c r="C15" s="37" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="20">
+    <row r="15" ht="15.6" customFormat="1" customHeight="1" s="29">
+      <c r="B15" s="85" t="n"/>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>Nutrition</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="n">
         <v>1.75</v>
       </c>
-      <c r="E15" s="21">
-        <v>0</v>
-      </c>
-      <c r="F15" s="22">
-        <v>0</v>
-      </c>
-      <c r="G15" s="39">
-        <v>0</v>
-      </c>
-      <c r="H15" s="24"/>
-      <c r="I15" s="43">
-        <v>0</v>
-      </c>
-      <c r="J15" s="32">
-        <v>0</v>
-      </c>
-      <c r="K15" s="24">
-        <v>0</v>
-      </c>
-      <c r="L15" s="2"/>
-      <c r="M15" s="28"/>
-      <c r="N15" s="28"/>
+      <c r="E15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="24" t="n"/>
+      <c r="I15" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="78" t="n"/>
+      <c r="M15" s="74" t="n"/>
+      <c r="N15" s="74" t="n"/>
     </row>
-    <row r="16" spans="2:14" s="29" customFormat="1" ht="15.45" customHeight="1" thickBot="1">
-      <c r="B16" s="64"/>
-      <c r="C16" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="45">
-        <v>0</v>
-      </c>
-      <c r="E16" s="46">
+    <row r="16" ht="15.45" customFormat="1" customHeight="1" s="29" thickBot="1">
+      <c r="B16" s="88" t="n"/>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>VCMA</t>
+        </is>
+      </c>
+      <c r="D16" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="46" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="47">
         <f>[1]Sheet1!$AS$18</f>
-        <v>0.1</v>
-      </c>
-      <c r="G16" s="48">
-        <v>0</v>
-      </c>
-      <c r="H16" s="36"/>
+        <v/>
+      </c>
+      <c r="G16" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="36" t="n"/>
       <c r="I16" s="49">
         <f>[1]Sheet1!$AS$21</f>
-        <v>0.1</v>
-      </c>
-      <c r="J16" s="35">
-        <v>0</v>
-      </c>
-      <c r="K16" s="36">
-        <v>0</v>
-      </c>
-      <c r="L16" s="2"/>
-      <c r="M16" s="28"/>
-      <c r="N16" s="28"/>
+        <v/>
+      </c>
+      <c r="J16" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="78" t="n"/>
+      <c r="M16" s="74" t="n"/>
+      <c r="N16" s="74" t="n"/>
     </row>
-    <row r="17" spans="2:28" s="54" customFormat="1">
-      <c r="B17" s="51"/>
-      <c r="C17" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="55">
-        <v>0.22556390977443608</v>
-      </c>
-      <c r="E17" s="55">
-        <v>0.18796992481203006</v>
-      </c>
-      <c r="F17" s="55">
-        <v>0.22556390977443608</v>
-      </c>
-      <c r="G17" s="55">
-        <v>0.22556390977443608</v>
-      </c>
-      <c r="H17" s="52"/>
-      <c r="I17" s="56">
-        <v>1.8796992481203006E-3</v>
-      </c>
-      <c r="J17" s="56">
-        <v>1.8796992481203006E-3</v>
-      </c>
-      <c r="K17" s="56">
-        <v>1.8796992481203006E-3</v>
-      </c>
-      <c r="L17" s="51"/>
-      <c r="M17" s="53"/>
-      <c r="N17" s="53"/>
-      <c r="O17" s="53"/>
-      <c r="P17" s="53"/>
-      <c r="Q17" s="53"/>
-      <c r="R17" s="53"/>
-      <c r="S17" s="53"/>
-      <c r="T17" s="53"/>
-      <c r="U17" s="53"/>
-      <c r="V17" s="53"/>
-      <c r="W17" s="53"/>
-      <c r="X17" s="53"/>
-      <c r="Y17" s="53"/>
-      <c r="Z17" s="53"/>
-      <c r="AA17" s="53"/>
-      <c r="AB17" s="53"/>
+    <row r="17" customFormat="1" s="54">
+      <c r="B17" s="51" t="n"/>
+      <c r="C17" s="52" t="inlineStr">
+        <is>
+          <t>per Program Target (target/13)</t>
+        </is>
+      </c>
+      <c r="D17" s="89" t="n">
+        <v>0.2255639097744361</v>
+      </c>
+      <c r="E17" s="89" t="n">
+        <v>0.1879699248120301</v>
+      </c>
+      <c r="F17" s="89" t="n">
+        <v>0.2255639097744361</v>
+      </c>
+      <c r="G17" s="89" t="n">
+        <v>0.2255639097744361</v>
+      </c>
+      <c r="H17" s="52" t="n"/>
+      <c r="I17" s="90" t="n">
+        <v>0.001879699248120301</v>
+      </c>
+      <c r="J17" s="90" t="n">
+        <v>0.001879699248120301</v>
+      </c>
+      <c r="K17" s="90" t="n">
+        <v>0.001879699248120301</v>
+      </c>
+      <c r="L17" s="51" t="n"/>
+      <c r="M17" s="91" t="n"/>
+      <c r="N17" s="91" t="n"/>
+      <c r="O17" s="91" t="n"/>
+      <c r="P17" s="91" t="n"/>
+      <c r="Q17" s="91" t="n"/>
+      <c r="R17" s="91" t="n"/>
+      <c r="S17" s="91" t="n"/>
+      <c r="T17" s="91" t="n"/>
+      <c r="U17" s="91" t="n"/>
+      <c r="V17" s="91" t="n"/>
+      <c r="W17" s="91" t="n"/>
+      <c r="X17" s="91" t="n"/>
+      <c r="Y17" s="91" t="n"/>
+      <c r="Z17" s="91" t="n"/>
+      <c r="AA17" s="91" t="n"/>
+      <c r="AB17" s="91" t="n"/>
     </row>
-    <row r="19" spans="2:28" hidden="1">
-      <c r="B19" s="57"/>
-      <c r="D19" s="58"/>
+    <row r="18"/>
+    <row r="19" hidden="1">
+      <c r="B19" s="57" t="n"/>
+      <c r="D19" s="58" t="n"/>
     </row>
-    <row r="20" spans="2:28" hidden="1">
-      <c r="B20" s="57"/>
-      <c r="D20" s="50"/>
+    <row r="20" hidden="1">
+      <c r="B20" s="57" t="n"/>
+      <c r="D20" s="50" t="n"/>
     </row>
-    <row r="21" spans="2:28" hidden="1">
-      <c r="B21" s="57"/>
-      <c r="D21" s="57"/>
+    <row r="21" hidden="1">
+      <c r="B21" s="57" t="n"/>
+      <c r="D21" s="57" t="n"/>
     </row>
-    <row r="22" spans="2:28" hidden="1"/>
-    <row r="23" spans="2:28" hidden="1"/>
+    <row r="22" hidden="1"/>
+    <row r="23" hidden="1"/>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="C1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="D2:H2"/>
     <mergeCell ref="B4:B7"/>
-    <mergeCell ref="B8:B11"/>
     <mergeCell ref="B12:B16"/>
-    <mergeCell ref="C1:K1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="I2:K2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:D16">
     <cfRule type="colorScale" priority="38">
@@ -2031,12 +2144,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="8" scale="88" orientation="landscape" r:id="rId1"/>
+  <pageSetup orientation="landscape" paperSize="8" scale="88"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{9d258917-277f-42cd-a3cd-14c4e9ee58bc}" enabled="1" method="Standard" siteId="{38ae3bcd-9579-4fd4-adda-b42e1495d55a}" contentBits="0" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>